<commit_message>
Simplify POS checkout UI
</commit_message>
<xml_diff>
--- a/outputs/beervibes.xlsx
+++ b/outputs/beervibes.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R4a9de67613d848bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="Ra30dca5e657345fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="3" r:id="Raa7444536e4041b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Logs" sheetId="4" r:id="R337de15d49e041ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="5" r:id="R0a358f78e3644b30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Raaac72b4b5e2452b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="Rb2e031a68f01470d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="3" r:id="Rd9a6bd3da6d84c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Logs" sheetId="4" r:id="R9e435881356d42d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="5" r:id="R939fce14a97b46cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -284,7 +284,7 @@
         <x:v>เบียร์ช้างขวด</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:f>Products!D2</x:f>
+        <x:f>Products!E2</x:f>
         <x:v>48</x:v>
       </x:c>
       <x:c r="F5" t="str"/>
@@ -294,7 +294,7 @@
         <x:v>Current Stock Units</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:f>SUM(Products!D2:D200)</x:f>
+        <x:f>SUM(Products!E2:E200)</x:f>
         <x:v>132</x:v>
       </x:c>
       <x:c r="C6" t="str"/>
@@ -302,7 +302,7 @@
         <x:v>เบียร์ลีโอขวด</x:v>
       </x:c>
       <x:c r="E6" t="n">
-        <x:f>Products!D3</x:f>
+        <x:f>Products!E3</x:f>
         <x:v>48</x:v>
       </x:c>
       <x:c r="F6" t="str"/>
@@ -320,7 +320,7 @@
         <x:v>เบียร์สิงห์ขวด</x:v>
       </x:c>
       <x:c r="E7" t="n">
-        <x:f>Products!D4</x:f>
+        <x:f>Products!E4</x:f>
         <x:v>36</x:v>
       </x:c>
       <x:c r="F7" t="str"/>
@@ -429,6 +429,7 @@
     <x:col min="4" max="4" width="15.5600004196167" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15.5600004196167" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="15.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15.5600004196167" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -442,12 +443,15 @@
         <x:v>price</x:v>
       </x:c>
       <x:c r="D1" t="str">
+        <x:v>cost</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
         <x:v>stock</x:v>
       </x:c>
-      <x:c r="E1" t="str">
+      <x:c r="F1" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="F1" t="str">
+      <x:c r="G1" t="str">
         <x:v>category</x:v>
       </x:c>
     </x:row>
@@ -462,12 +466,15 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="D2" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E2" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="E2" s="1" t="b">
+      <x:c r="F2" s="1" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F2" t="str">
+      <x:c r="G2" t="str">
         <x:v>Beer</x:v>
       </x:c>
     </x:row>
@@ -482,12 +489,15 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="D3" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E3" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="E3" s="1" t="b">
+      <x:c r="F3" s="1" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F3" t="str">
+      <x:c r="G3" t="str">
         <x:v>Beer</x:v>
       </x:c>
     </x:row>
@@ -502,12 +512,15 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="D4" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E4" t="n">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="E4" s="1" t="b">
+      <x:c r="F4" s="1" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F4" t="str">
+      <x:c r="G4" t="str">
         <x:v>Beer</x:v>
       </x:c>
     </x:row>
@@ -529,7 +542,9 @@
     <x:col min="7" max="7" width="17.780000686645508" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="17.780000686645508" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="17.780000686645508" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="28.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="28.889999389648438" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -561,6 +576,12 @@
         <x:v>total_amount</x:v>
       </x:c>
       <x:c r="J1" t="str">
+        <x:v>total_cost</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>gross_profit</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
         <x:v>items_json</x:v>
       </x:c>
     </x:row>

</xml_diff>